<commit_message>
Fix overdue logic, SLA formula, date format, and card alignment
- Overdue: now includes open tasks (elapsed > target OR past SLAAdjustedDate) AND closed tasks (TotalHoursOnTask > SLAInHours OR DateCompleted > SLAAdjustedDate)
- SLA compliance: canonical formula (TotalHoursOnTask <> 0 AND < SLAInHours) OR (DateCompleted <= SLAAdjustedDate)
- Task codes query: removed Tasks JOIN fan-out; now returns correct 3094 rows
- Drill-through date columns: format changed to dd/mm/yyyy with hh:mm:ss on second line; font size 12px matching task-id style
- Team cards: Overdue value right-aligned with paddingRight 20px
- Tooltips: updated overdue and SLA tooltips to reflect canonical logic
- CLAUDE.md: updated SLA and overdue definitions
</commit_message>
<xml_diff>
--- a/docs/SLA_Dashboard_Format Details .xlsx
+++ b/docs/SLA_Dashboard_Format Details .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mortgageezy-my.sharepoint.com/personal/ntruong_mezy_com_au/Documents/Project_VibeCoding/SLA Dashboard/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A6B08A9D-CDB2-4330-8D50-DA304FD8BC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671C2245-EA5A-4F16-A2D7-51C667107410}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{A6B08A9D-CDB2-4330-8D50-DA304FD8BC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00F58EFB-E2D3-4952-B2EB-D741982FDB39}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7E3D69AE-E9EC-49D5-8FB9-D5729AE146C8}"/>
+    <workbookView minimized="1" xWindow="30330" yWindow="1380" windowWidth="24690" windowHeight="12525" xr2:uid="{7E3D69AE-E9EC-49D5-8FB9-D5729AE146C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1752" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1752" uniqueCount="563">
   <si>
     <t>Typography Audit — SLA Performance Dashboard</t>
   </si>
@@ -2669,6 +2669,18 @@
   </si>
   <si>
     <t>Weright var 600</t>
+  </si>
+  <si>
+    <t>20 px</t>
+  </si>
+  <si>
+    <t>9PX</t>
+  </si>
+  <si>
+    <t>9px</t>
+  </si>
+  <si>
+    <t>9 px</t>
   </si>
 </sst>
 </file>
@@ -4929,10 +4941,10 @@
         <v>46</v>
       </c>
       <c r="F63" s="31" t="s">
-        <v>542</v>
+        <v>562</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>86</v>
+        <v>561</v>
       </c>
       <c r="H63" s="3">
         <v>500</v>
@@ -5037,7 +5049,7 @@
         <v>541</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>56</v>
+        <v>560</v>
       </c>
       <c r="H66" s="3">
         <v>500</v>
@@ -5072,7 +5084,7 @@
         <v>541</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>56</v>
+        <v>560</v>
       </c>
       <c r="H67" s="3">
         <v>500</v>
@@ -5107,7 +5119,7 @@
         <v>541</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>56</v>
+        <v>560</v>
       </c>
       <c r="H68" s="3">
         <v>500</v>
@@ -5142,7 +5154,7 @@
         <v>541</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>79</v>
+        <v>559</v>
       </c>
       <c r="H69" s="3">
         <v>600</v>
@@ -5177,7 +5189,7 @@
         <v>541</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>79</v>
+        <v>559</v>
       </c>
       <c r="H70" s="3">
         <v>600</v>
@@ -5212,7 +5224,7 @@
         <v>541</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>79</v>
+        <v>559</v>
       </c>
       <c r="H71" s="3">
         <v>600</v>
@@ -10915,5 +10927,6 @@
     <hyperlink ref="I236" r:id="rId114" display="vscode-file://vscode-app/c:/Users/Ngoc/AppData/Local/Programs/Microsoft VS Code/8761a5560c/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{8A65A4D2-554A-400F-B827-5FD50A6CC78A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId115"/>
 </worksheet>
 </file>
</xml_diff>